<commit_message>
limpieza en el código principal
</commit_message>
<xml_diff>
--- a/proyeccion_futura_sbs.xlsx
+++ b/proyeccion_futura_sbs.xlsx
@@ -64,14 +64,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>7.210000038146973</v>
+        <v>6.809999942779541</v>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>9.300000190734863</v>
+        <v>8.989999771118164</v>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
@@ -581,11 +581,11 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>8.729999542236328</v>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>AA-</t>
+        <v>8.180000305175781</v>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>A+</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>9.390000343322754</v>
+        <v>8.670000076293945</v>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
@@ -623,7 +623,7 @@
       <c r="C6" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>AAA</t>
         </is>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>6.699999809265137</v>
+        <v>6.949999809265137</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
@@ -661,11 +661,11 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>8.520000457763672</v>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>AA-</t>
+        <v>8.310000419616699</v>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>A+</t>
         </is>
       </c>
     </row>
@@ -681,9 +681,9 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>8.060000419616699</v>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
+        <v>7.679999828338623</v>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>A+</t>
         </is>
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>9.25</v>
+        <v>8.949999809265137</v>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>8.619999885559082</v>
+        <v>8.779999732971191</v>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>6</v>
+        <v>6.340000152587891</v>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
@@ -761,11 +761,11 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>AA-</t>
+        <v>7.630000114440918</v>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>A+</t>
         </is>
       </c>
     </row>
@@ -781,11 +781,11 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+        <v>7.800000190734863</v>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>A+</t>
         </is>
       </c>
     </row>
@@ -801,11 +801,11 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>8.260000228881836</v>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>A+</t>
+        <v>7.480000019073486</v>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>9.270000457763672</v>
+        <v>8.920000076293945</v>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>7.46999979019165</v>
+        <v>7.070000171661377</v>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
@@ -861,11 +861,11 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>9.439999580383301</v>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>AA-</t>
+        <v>8.390000343322754</v>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>A+</t>
         </is>
       </c>
     </row>
@@ -881,11 +881,11 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>7.880000114440918</v>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>A+</t>
+        <v>6.989999771118164</v>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -901,11 +901,11 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>6.920000076293945</v>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+        <v>6.21999979019165</v>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>A-</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>8.770000457763672</v>
+        <v>9.159999847412109</v>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>

</xml_diff>